<commit_message>
Fix wrong expected values found in review; label answer cells
- week4 Step2: RSS_left/RSS_right/Total RSS for splits s=1.5, 4.5, 5.5 were
  incorrect (best split s=2.5 unaffected); answer key updated to
  38.8 / 5.5 / 22.67 / 37.5 / 53.2
- week3 Step2: bootstrap SE corrected 1.0116 -> 1.01105 (correct answers
  were marked wrong at 3-decimal rounding)
- all worksheets: answer rows now carry an explicit 'Your Answer:' label
- re-verified: LibreOffice recalc zero errors; fill-answers self-test passes
  all 202 checks across the 7 workbooks
</commit_message>
<xml_diff>
--- a/week1/homework-test-error-knn.xlsx
+++ b/week1/homework-test-error-knn.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="112">
   <si>
     <t xml:space="preserve">[Description] Test Error, Bias–Variance &amp; KNN</t>
   </si>
@@ -132,6 +132,9 @@
   </si>
   <si>
     <t xml:space="preserve">SUM of column (yᵢ-ŷA)² / 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your Answer:</t>
   </si>
   <si>
     <t xml:space="preserve">Train MSE, Model B =</t>
@@ -518,60 +521,56 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -844,114 +843,114 @@
   <dimension ref="A1:B29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="5" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="5" t="s">
         <v>21</v>
       </c>
     </row>
@@ -971,333 +970,343 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="9" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="10" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
+      <c r="A12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="7" t="n">
         <v>3.5</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="6" t="str">
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="5" t="str">
         <f aca="false">IF(COUNT(E12:F12)=0,"",IF(AND(ROUND(E12,3)=ROUND(0.25,3),ROUND(F12,3)=ROUND(0,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="n">
+      <c r="A13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="7" t="n">
         <v>4.5</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="6" t="str">
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="5" t="str">
         <f aca="false">IF(COUNT(E13:F13)=0,"",IF(AND(ROUND(E13,3)=ROUND(0.25,3),ROUND(F13,3)=ROUND(0,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
+      <c r="A14" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="6" t="str">
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="5" t="str">
         <f aca="false">IF(COUNT(E14:F14)=0,"",IF(AND(ROUND(E14,3)=ROUND(1,3),ROUND(F14,3)=ROUND(0,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="n">
+      <c r="A15" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="7" t="n">
         <v>5.5</v>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="6" t="str">
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="5" t="str">
         <f aca="false">IF(COUNT(E15:F15)=0,"",IF(AND(ROUND(E15,3)=ROUND(0.25,3),ROUND(F15,3)=ROUND(0,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="n">
+      <c r="A16" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="7" t="n">
         <v>6.5</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="6" t="str">
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="5" t="str">
         <f aca="false">IF(COUNT(E16:F16)=0,"",IF(AND(ROUND(E16,3)=ROUND(0.25,3),ROUND(F16,3)=ROUND(0,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="D18" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="6" t="str">
-        <f aca="false">IF(F18="","",IF(ROUND(F18,3)=ROUND(0.4,3),"✓","✗"))</f>
+      <c r="E18" s="11"/>
+      <c r="F18" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G18" s="12"/>
+      <c r="H18" s="5" t="str">
+        <f aca="false">IF(G18="","",IF(ROUND(G18,3)=ROUND(0.4,3),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="11"/>
+      <c r="F20" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="6" t="str">
-        <f aca="false">IF(F20="","",IF(ROUND(F20,3)=ROUND(0,3),"✓","✗"))</f>
+      <c r="G20" s="12"/>
+      <c r="H20" s="5" t="str">
+        <f aca="false">IF(G20="","",IF(ROUND(G20,3)=ROUND(0,3),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>38</v>
+      <c r="A22" s="4" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="E24" s="11" t="s">
+      <c r="E24" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="F24" s="11" t="s">
+      <c r="F24" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="10" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="n">
+      <c r="A25" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B25" s="8" t="n">
+      <c r="B25" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C25" s="8" t="n">
+      <c r="C25" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="D25" s="8" t="n">
+      <c r="D25" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="6" t="str">
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="5" t="str">
         <f aca="false">IF(COUNT(E25:F25)=0,"",IF(AND(ROUND(E25,3)=ROUND(4,3),ROUND(F25,3)=ROUND(16,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="n">
+      <c r="A26" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B26" s="8" t="n">
+      <c r="B26" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="C26" s="8" t="n">
+      <c r="C26" s="7" t="n">
         <v>7.5</v>
       </c>
-      <c r="D26" s="8" t="n">
+      <c r="D26" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="6" t="str">
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="5" t="str">
         <f aca="false">IF(COUNT(E26:F26)=0,"",IF(AND(ROUND(E26,3)=ROUND(2.25,3),ROUND(F26,3)=ROUND(4,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="n">
+      <c r="A27" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B27" s="8" t="n">
+      <c r="B27" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="C27" s="8" t="n">
+      <c r="C27" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="D27" s="8" t="n">
+      <c r="D27" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="6" t="str">
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="5" t="str">
         <f aca="false">IF(COUNT(E27:F27)=0,"",IF(AND(ROUND(E27,3)=ROUND(0,3),ROUND(F27,3)=ROUND(4,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C29" s="12" t="s">
+      <c r="A29" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="6" t="str">
-        <f aca="false">IF(F29="","",IF(ROUND(F29,3)=ROUND(2.083333,3),"✓","✗"))</f>
+      <c r="D29" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E29" s="11"/>
+      <c r="F29" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G29" s="12"/>
+      <c r="H29" s="5" t="str">
+        <f aca="false">IF(G29="","",IF(ROUND(G29,3)=ROUND(2.083333,3),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D31" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C31" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="6" t="str">
-        <f aca="false">IF(F31="","",IF(ROUND(F31,3)=ROUND(8,3),"✓","✗"))</f>
+      <c r="E31" s="11"/>
+      <c r="F31" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G31" s="12"/>
+      <c r="H31" s="5" t="str">
+        <f aca="false">IF(G31="","",IF(ROUND(G31,3)=ROUND(8,3),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C33" s="12" t="s">
+      <c r="A33" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="6" t="str">
-        <f aca="false">IF(F33="","",IF(UPPER(TRIM(F33))=UPPER("B"),"✓","✗"))</f>
+      <c r="D33" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E33" s="11"/>
+      <c r="F33" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G33" s="12"/>
+      <c r="H33" s="5" t="str">
+        <f aca="false">IF(G33="","",IF(UPPER(TRIM(G33))=UPPER("B"),"✓","✗"))</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D33:E33"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:J33">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -1322,151 +1331,155 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>44</v>
+      <c r="A1" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>45</v>
+      <c r="A3" s="2" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
-        <v>46</v>
+      <c r="A5" s="9" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>47</v>
+      <c r="A7" s="5" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>48</v>
+      <c r="A9" s="4" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="C11" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="D11" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="E11" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B12" s="8" t="n">
+      <c r="A12" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="6" t="str">
+      <c r="E12" s="8"/>
+      <c r="F12" s="5" t="str">
         <f aca="false">IF(COUNT(E12)=0,"",IF(AND(ROUND(E12,3)=ROUND(5.5,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B13" s="8" t="n">
+      <c r="A13" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="6" t="str">
+      <c r="E13" s="8"/>
+      <c r="F13" s="5" t="str">
         <f aca="false">IF(COUNT(E13)=0,"",IF(AND(ROUND(E13,3)=ROUND(3,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="B14" s="8" t="n">
+      <c r="A14" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="6" t="str">
+      <c r="E14" s="8"/>
+      <c r="F14" s="5" t="str">
         <f aca="false">IF(COUNT(E14)=0,"",IF(AND(ROUND(E14,3)=ROUND(4.5,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C16" s="12" t="s">
+      <c r="A16" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="6" t="str">
-        <f aca="false">IF(F16="","",IF(UPPER(TRIM(F16))=UPPER("Medium"),"✓","✗"))</f>
+      <c r="D16" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="E16" s="11"/>
+      <c r="F16" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G16" s="12"/>
+      <c r="H16" s="5" t="str">
+        <f aca="false">IF(G16="","",IF(UPPER(TRIM(G16))=UPPER("Medium"),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C18" s="12" t="s">
+      <c r="A18" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="6" t="str">
-        <f aca="false">IF(F18="","",IF(ROUND(F18,3)=ROUND(1,3),"✓","✗"))</f>
+      <c r="D18" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="E18" s="11"/>
+      <c r="F18" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G18" s="12"/>
+      <c r="H18" s="5" t="str">
+        <f aca="false">IF(G18="","",IF(ROUND(G18,3)=ROUND(1,3),"✓","✗"))</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D18:E18"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:J18">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -1491,243 +1504,249 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>61</v>
+      <c r="A1" s="1" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>62</v>
+      <c r="A3" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
-        <v>63</v>
+      <c r="A5" s="9" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>64</v>
+      <c r="A7" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>65</v>
+      <c r="A9" s="4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="C11" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="D11" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="E11" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="F11" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
+      <c r="A12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="6" t="str">
+      <c r="D12" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="5" t="str">
         <f aca="false">IF(COUNT(E12:F12)=0,"",IF(AND(ROUND(E12,3)=ROUND(5,3),ROUND(F12,3)=ROUND(4,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="n">
+      <c r="A13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="6" t="str">
+      <c r="D13" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="5" t="str">
         <f aca="false">IF(COUNT(E13:F13)=0,"",IF(AND(ROUND(E13,3)=ROUND(1,3),ROUND(F13,3)=ROUND(1,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
+      <c r="A14" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="5" t="str">
+        <f aca="false">IF(COUNT(E14:F14)=0,"",IF(AND(ROUND(E14,3)=ROUND(2,3),ROUND(F14,3)=ROUND(2,3)),"✓","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="5" t="str">
+        <f aca="false">IF(COUNT(E15:F15)=0,"",IF(AND(ROUND(E15,3)=ROUND(8,3),ROUND(F15,3)=ROUND(5.5,3)),"✓","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="6" t="str">
-        <f aca="false">IF(COUNT(E14:F14)=0,"",IF(AND(ROUND(E14,3)=ROUND(2,3),ROUND(F14,3)=ROUND(2,3)),"✓","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B15" s="8" t="n">
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="5" t="str">
+        <f aca="false">IF(COUNT(E16:F16)=0,"",IF(AND(ROUND(E16,3)=ROUND(4,3),ROUND(F16,3)=ROUND(3,3)),"✓","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="6" t="str">
-        <f aca="false">IF(COUNT(E15:F15)=0,"",IF(AND(ROUND(E15,3)=ROUND(8,3),ROUND(F15,3)=ROUND(5.5,3)),"✓","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="n">
+      <c r="C17" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="6" t="str">
-        <f aca="false">IF(COUNT(E16:F16)=0,"",IF(AND(ROUND(E16,3)=ROUND(4,3),ROUND(F16,3)=ROUND(3,3)),"✓","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="6" t="str">
+      <c r="D17" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="5" t="str">
         <f aca="false">IF(COUNT(E17:F17)=0,"",IF(AND(ROUND(E17,3)=ROUND(8,3),ROUND(F17,3)=ROUND(5.5,3)),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>73</v>
+      <c r="A19" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>74</v>
+      <c r="A21" s="4" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="C23" s="12" t="s">
+      <c r="A23" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="6" t="str">
-        <f aca="false">IF(F23="","",IF(UPPER(TRIM(F23))=UPPER("Blue"),"✓","✗"))</f>
+      <c r="D23" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="E23" s="11"/>
+      <c r="F23" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G23" s="12"/>
+      <c r="H23" s="5" t="str">
+        <f aca="false">IF(G23="","",IF(UPPER(TRIM(G23))=UPPER("Blue"),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C25" s="12" t="s">
+      <c r="A25" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="6" t="str">
-        <f aca="false">IF(F25="","",IF(ROUND(F25,3)=ROUND(0.666667,3),"✓","✗"))</f>
+      <c r="D25" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E25" s="11"/>
+      <c r="F25" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G25" s="12"/>
+      <c r="H25" s="5" t="str">
+        <f aca="false">IF(G25="","",IF(ROUND(G25,3)=ROUND(0.666667,3),"✓","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C27" s="12" t="s">
+      <c r="A27" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="6" t="str">
-        <f aca="false">IF(F27="","",IF(UPPER(TRIM(F27))=UPPER("Blue"),"✓","✗"))</f>
+      <c r="D27" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="E27" s="11"/>
+      <c r="F27" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G27" s="12"/>
+      <c r="H27" s="5" t="str">
+        <f aca="false">IF(G27="","",IF(UPPER(TRIM(G27))=UPPER("Blue"),"✓","✗"))</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D27:E27"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:J27">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -1755,161 +1774,161 @@
   <dimension ref="A1:B28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>81</v>
+      <c r="A1" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>82</v>
+      <c r="A3" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>83</v>
+      <c r="A5" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="B7" s="8" t="n">
+      <c r="A7" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="7" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B8" s="8" t="n">
+      <c r="A8" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" s="7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B9" s="8" t="n">
+      <c r="A9" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" s="7" t="n">
         <v>2.0833</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="B10" s="8" t="n">
+      <c r="A10" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" s="7" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="B11" s="8" t="s">
+      <c r="A11" s="5" t="s">
         <v>89</v>
       </c>
+      <c r="B11" s="7" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B12" s="8" t="s">
+      <c r="A12" s="5" t="s">
         <v>91</v>
       </c>
+      <c r="B12" s="7" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B13" s="8" t="s">
+      <c r="A13" s="5" t="s">
         <v>93</v>
       </c>
+      <c r="B13" s="7" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B14" s="8" t="s">
+      <c r="A14" s="5" t="s">
         <v>95</v>
       </c>
+      <c r="B14" s="7" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
-        <v>96</v>
+      <c r="A16" s="4" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="B18" s="8" t="s">
+      <c r="A18" s="5" t="s">
         <v>98</v>
       </c>
+      <c r="B18" s="7" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="B19" s="8" t="s">
+      <c r="A19" s="5" t="s">
         <v>100</v>
       </c>
+      <c r="B19" s="7" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B20" s="8" t="n">
+      <c r="A20" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" s="7" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>102</v>
+      <c r="A22" s="4" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B24" s="8" t="s">
+      <c r="A24" s="5" t="s">
         <v>104</v>
       </c>
+      <c r="B24" s="7" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B25" s="8" t="s">
+      <c r="A25" s="5" t="s">
         <v>106</v>
       </c>
+      <c r="B25" s="7" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>71</v>
+      <c r="A26" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="B27" s="8" t="s">
+      <c r="A27" s="5" t="s">
         <v>109</v>
       </c>
+      <c r="B27" s="7" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>71</v>
+      <c r="A28" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>